<commit_message>
Orden de fichero netejaS
</commit_message>
<xml_diff>
--- a/data/netejaS.xlsx
+++ b/data/netejaS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\_Flask_Python\gepV\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{057BBD91-4957-4929-A2F0-C488D57F6F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F501530E-1570-4595-98D4-7764F1525918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28692" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{E7BEF806-E2E7-45EE-9B5C-D08728AB8555}"/>
   </bookViews>
@@ -135,10 +135,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="d\-m;@"/>
+    <numFmt numFmtId="165" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,6 +180,13 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -293,41 +301,24 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="1" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -336,47 +327,20 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="4" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="4" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="1" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="1" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="1" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -390,9 +354,57 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="9" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="6" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="10" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="9" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -803,12 +815,14 @@
   <cols>
     <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" style="13"/>
+    <col min="3" max="3" width="11.5546875" style="7"/>
     <col min="4" max="4" width="40" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.5546875" style="34"/>
+    <col min="7" max="7" width="11.5546875" style="42"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="22" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -820,1324 +834,1324 @@
       <c r="D1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="35" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="3">
         <v>46076</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="27">
         <v>0.36458333333333331</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="27">
         <v>0.39583333333333331</v>
       </c>
-      <c r="G2" s="8">
+      <c r="G2" s="36">
         <v>3.125E-2</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="3">
         <v>46076</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="27">
         <v>0.39583333333333331</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="27">
         <v>0.42708333333333331</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="36">
         <v>3.125E-2</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="12">
         <v>46076</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="22">
+      <c r="E4" s="28">
         <v>0.41666666666666669</v>
       </c>
-      <c r="F4" s="22">
+      <c r="F4" s="28">
         <v>0.47916666666666669</v>
       </c>
-      <c r="G4" s="23">
+      <c r="G4" s="37">
         <v>6.25E-2</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="12">
         <v>46076</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="28">
         <v>0.47916666666666669</v>
       </c>
-      <c r="F5" s="22">
+      <c r="F5" s="28">
         <v>0.52083333333333337</v>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="37">
         <v>4.1666666666666685E-2</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="9">
         <v>46076</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="29">
         <v>0.59375</v>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="29">
         <v>0.63541666666666663</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="38">
         <v>4.166666666666663E-2</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="15">
         <v>46076</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="D7" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="28">
+      <c r="E7" s="30">
         <v>0.625</v>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="30">
         <v>0.68055555555555558</v>
       </c>
-      <c r="G7" s="29">
+      <c r="G7" s="39">
         <v>5.555555555555558E-2</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="15">
+      <c r="C8" s="9">
         <v>46076</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="29">
         <v>0.63541666666666663</v>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="29">
         <v>0.68055555555555558</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="38">
         <v>4.5138888888888951E-2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="15">
+      <c r="C9" s="9">
         <v>46076</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="29">
         <v>0.6875</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="29">
         <v>0.83333333333333337</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="38">
         <v>0.14583333333333337</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="39" t="s">
+      <c r="A10" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="15">
         <v>46076</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="30">
         <v>0.6875</v>
       </c>
-      <c r="F10" s="28">
+      <c r="F10" s="30">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G10" s="29">
+      <c r="G10" s="39">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="3">
         <v>46076</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="27">
         <v>0.6875</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="27">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="36">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="12">
         <v>46076</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="28">
         <v>0.69791666666666663</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="28">
         <v>0.84375</v>
       </c>
-      <c r="G12" s="23">
+      <c r="G12" s="37">
         <v>0.14583333333333326</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="40" t="s">
+      <c r="A13" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="5">
         <v>46076</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="31">
         <v>0.72916666666666663</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="31">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="40">
         <v>0.125</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="39" t="s">
+      <c r="A14" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="9">
         <v>46076</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E14" s="17">
+      <c r="E14" s="29">
         <v>0.84027777777777779</v>
       </c>
-      <c r="F14" s="17">
+      <c r="F14" s="29">
         <v>0.89236111111111116</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="38">
         <v>5.208333333333337E-2</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="3">
         <v>46077</v>
       </c>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="E15" s="35">
+      <c r="E15" s="32">
         <v>0.46875</v>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="32">
         <v>0.5</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="36">
         <v>3.125E-2</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="15">
         <v>46077</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="28">
+      <c r="E16" s="30">
         <v>0.60069444444444442</v>
       </c>
-      <c r="F16" s="28">
+      <c r="F16" s="30">
         <v>0.68055555555555558</v>
       </c>
-      <c r="G16" s="29">
+      <c r="G16" s="39">
         <v>7.986111111111116E-2</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="38" t="s">
+      <c r="A17" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="12">
         <v>46077</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="D17" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="28">
         <v>0.61111111111111116</v>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="28">
         <v>0.65277777777777779</v>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="41">
         <v>4.166666666666663E-2</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="15">
+      <c r="C18" s="9">
         <v>46077</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="D18" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E18" s="17">
+      <c r="E18" s="29">
         <v>0.63541666666666663</v>
       </c>
-      <c r="F18" s="17">
+      <c r="F18" s="29">
         <v>0.68055555555555558</v>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="38">
         <v>4.5138888888888951E-2</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="39" t="s">
+      <c r="A19" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="20">
+      <c r="C19" s="12">
         <v>46077</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="D19" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="E19" s="22">
+      <c r="E19" s="28">
         <v>0.65277777777777779</v>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="28">
         <v>0.70138888888888884</v>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="41">
         <v>4.8611111111111049E-2</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="15">
+      <c r="C20" s="9">
         <v>46077</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="29">
         <v>0.6875</v>
       </c>
-      <c r="F20" s="17">
+      <c r="F20" s="29">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="38">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="39" t="s">
+      <c r="A21" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="26">
+      <c r="C21" s="15">
         <v>46077</v>
       </c>
-      <c r="D21" s="27" t="s">
+      <c r="D21" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="E21" s="28">
+      <c r="E21" s="30">
         <v>0.6875</v>
       </c>
-      <c r="F21" s="28">
+      <c r="F21" s="30">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G21" s="29">
+      <c r="G21" s="39">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="38" t="s">
+      <c r="A22" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="33" t="s">
+      <c r="B22" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="3">
         <v>46077</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E22" s="7">
+      <c r="E22" s="27">
         <v>0.6875</v>
       </c>
-      <c r="F22" s="7">
+      <c r="F22" s="27">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="36">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="12">
         <v>46077</v>
       </c>
-      <c r="D23" s="21" t="s">
+      <c r="D23" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="22">
+      <c r="E23" s="28">
         <v>0.70833333333333337</v>
       </c>
-      <c r="F23" s="22">
+      <c r="F23" s="28">
         <v>0.84375</v>
       </c>
-      <c r="G23" s="24">
+      <c r="G23" s="41">
         <v>0.13541666666666663</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="40" t="s">
+      <c r="A24" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="5">
         <v>46077</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="31">
         <v>0.72916666666666663</v>
       </c>
-      <c r="F24" s="11">
+      <c r="F24" s="31">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G24" s="12">
+      <c r="G24" s="40">
         <v>0.125</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="39" t="s">
+      <c r="A25" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="33" t="s">
+      <c r="B25" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="3">
         <v>46078</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="27">
         <v>0.5</v>
       </c>
-      <c r="F25" s="7">
+      <c r="F25" s="27">
         <v>0.58333333333333337</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="36">
         <v>8.333333333333337E-2</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="38" t="s">
+      <c r="A26" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="15">
+      <c r="C26" s="9">
         <v>46078</v>
       </c>
-      <c r="D26" s="16" t="s">
+      <c r="D26" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E26" s="17">
+      <c r="E26" s="29">
         <v>0.60763888888888884</v>
       </c>
-      <c r="F26" s="17">
+      <c r="F26" s="29">
         <v>0.63541666666666663</v>
       </c>
-      <c r="G26" s="18">
+      <c r="G26" s="38">
         <v>2.777777777777779E-2</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="39" t="s">
+      <c r="A27" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="12">
         <v>46078</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="E27" s="22">
+      <c r="E27" s="28">
         <v>0.61111111111111116</v>
       </c>
-      <c r="F27" s="22">
+      <c r="F27" s="28">
         <v>0.65277777777777779</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="41">
         <v>4.166666666666663E-2</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="39" t="s">
+      <c r="A28" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="15">
+      <c r="C28" s="9">
         <v>46078</v>
       </c>
-      <c r="D28" s="16" t="s">
+      <c r="D28" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E28" s="17">
+      <c r="E28" s="29">
         <v>0.63541666666666663</v>
       </c>
-      <c r="F28" s="17">
+      <c r="F28" s="29">
         <v>0.68055555555555558</v>
       </c>
-      <c r="G28" s="18">
+      <c r="G28" s="38">
         <v>4.5138888888888951E-2</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="38" t="s">
+      <c r="A29" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="20">
+      <c r="C29" s="12">
         <v>46078</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="D29" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="22">
+      <c r="E29" s="28">
         <v>0.65277777777777779</v>
       </c>
-      <c r="F29" s="22">
+      <c r="F29" s="28">
         <v>0.70138888888888884</v>
       </c>
-      <c r="G29" s="24">
+      <c r="G29" s="41">
         <v>4.8611111111111049E-2</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="38" t="s">
+      <c r="A30" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B30" s="25" t="s">
+      <c r="B30" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C30" s="26">
+      <c r="C30" s="15">
         <v>46078</v>
       </c>
-      <c r="D30" s="27" t="s">
+      <c r="D30" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E30" s="28">
+      <c r="E30" s="30">
         <v>0.65277777777777779</v>
       </c>
-      <c r="F30" s="28">
+      <c r="F30" s="30">
         <v>0.68402777777777779</v>
       </c>
-      <c r="G30" s="29">
+      <c r="G30" s="39">
         <v>3.125E-2</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="38" t="s">
+      <c r="A31" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B31" s="14" t="s">
+      <c r="B31" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="9">
         <v>46078</v>
       </c>
-      <c r="D31" s="16" t="s">
+      <c r="D31" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E31" s="17">
+      <c r="E31" s="29">
         <v>0.6875</v>
       </c>
-      <c r="F31" s="17">
+      <c r="F31" s="29">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G31" s="18">
+      <c r="G31" s="38">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="39" t="s">
+      <c r="A32" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="25" t="s">
+      <c r="B32" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C32" s="26">
+      <c r="C32" s="15">
         <v>46078</v>
       </c>
-      <c r="D32" s="27" t="s">
+      <c r="D32" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="E32" s="28">
+      <c r="E32" s="30">
         <v>0.6875</v>
       </c>
-      <c r="F32" s="28">
+      <c r="F32" s="30">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G32" s="29">
+      <c r="G32" s="39">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="38" t="s">
+      <c r="A33" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B33" s="33" t="s">
+      <c r="B33" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="5">
+      <c r="C33" s="3">
         <v>46078</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E33" s="7">
+      <c r="E33" s="27">
         <v>0.6875</v>
       </c>
-      <c r="F33" s="7">
+      <c r="F33" s="27">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G33" s="8">
+      <c r="G33" s="36">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="39" t="s">
+      <c r="A34" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="19" t="s">
+      <c r="B34" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C34" s="20">
+      <c r="C34" s="12">
         <v>46078</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="D34" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E34" s="22">
+      <c r="E34" s="28">
         <v>0.70833333333333337</v>
       </c>
-      <c r="F34" s="22">
+      <c r="F34" s="28">
         <v>0.84375</v>
       </c>
-      <c r="G34" s="24">
+      <c r="G34" s="41">
         <v>0.13541666666666663</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="40" t="s">
+      <c r="A35" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="36" t="s">
+      <c r="B35" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="9">
+      <c r="C35" s="5">
         <v>46078</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E35" s="11">
+      <c r="E35" s="31">
         <v>0.72916666666666663</v>
       </c>
-      <c r="F35" s="11">
+      <c r="F35" s="31">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G35" s="12">
+      <c r="G35" s="40">
         <v>0.125</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="39" t="s">
+      <c r="A36" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B36" s="33" t="s">
+      <c r="B36" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="5">
+      <c r="C36" s="3">
         <v>46079</v>
       </c>
-      <c r="D36" s="34" t="s">
+      <c r="D36" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="E36" s="35">
+      <c r="E36" s="32">
         <v>0.41666666666666669</v>
       </c>
-      <c r="F36" s="35">
+      <c r="F36" s="32">
         <v>0.46875</v>
       </c>
-      <c r="G36" s="8">
+      <c r="G36" s="36">
         <v>5.2083333333333315E-2</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="38" t="s">
+      <c r="A37" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B37" s="33" t="s">
+      <c r="B37" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C37" s="3">
         <v>46079</v>
       </c>
-      <c r="D37" s="34" t="s">
+      <c r="D37" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="E37" s="35">
+      <c r="E37" s="32">
         <v>0.41666666666666669</v>
       </c>
-      <c r="F37" s="35">
+      <c r="F37" s="32">
         <v>0.45833333333333331</v>
       </c>
-      <c r="G37" s="8">
+      <c r="G37" s="36">
         <v>4.166666666666663E-2</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="38" t="s">
+      <c r="A38" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="25" t="s">
+      <c r="B38" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C38" s="26">
+      <c r="C38" s="15">
         <v>46079</v>
       </c>
-      <c r="D38" s="30" t="s">
+      <c r="D38" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="E38" s="31">
+      <c r="E38" s="33">
         <v>0.59722222222222221</v>
       </c>
-      <c r="F38" s="31">
+      <c r="F38" s="33">
         <v>0.62847222222222221</v>
       </c>
-      <c r="G38" s="29">
+      <c r="G38" s="39">
         <v>3.125E-2</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="38" t="s">
+      <c r="A39" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B39" s="19" t="s">
+      <c r="B39" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C39" s="20">
+      <c r="C39" s="12">
         <v>46079</v>
       </c>
-      <c r="D39" s="21" t="s">
+      <c r="D39" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="E39" s="22">
+      <c r="E39" s="28">
         <v>0.60416666666666663</v>
       </c>
-      <c r="F39" s="22">
+      <c r="F39" s="28">
         <v>0.65972222222222221</v>
       </c>
-      <c r="G39" s="24">
+      <c r="G39" s="41">
         <v>5.555555555555558E-2</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="39" t="s">
+      <c r="A40" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B40" s="25" t="s">
+      <c r="B40" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C40" s="26">
+      <c r="C40" s="15">
         <v>46079</v>
       </c>
-      <c r="D40" s="32" t="s">
+      <c r="D40" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="E40" s="28">
+      <c r="E40" s="30">
         <v>0.62847222222222221</v>
       </c>
-      <c r="F40" s="28">
+      <c r="F40" s="30">
         <v>0.67708333333333337</v>
       </c>
-      <c r="G40" s="29">
+      <c r="G40" s="39">
         <v>4.861111111111116E-2</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="39" t="s">
+      <c r="A41" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B41" s="14" t="s">
+      <c r="B41" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C41" s="15">
+      <c r="C41" s="9">
         <v>46079</v>
       </c>
-      <c r="D41" s="16" t="s">
+      <c r="D41" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E41" s="17">
+      <c r="E41" s="29">
         <v>0.63541666666666663</v>
       </c>
-      <c r="F41" s="17">
+      <c r="F41" s="29">
         <v>0.68055555555555558</v>
       </c>
-      <c r="G41" s="18">
+      <c r="G41" s="38">
         <v>4.5138888888888951E-2</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="39" t="s">
+      <c r="A42" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B42" s="19" t="s">
+      <c r="B42" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C42" s="20">
+      <c r="C42" s="12">
         <v>46079</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="D42" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="E42" s="22">
+      <c r="E42" s="28">
         <v>0.65972222222222221</v>
       </c>
-      <c r="F42" s="22">
+      <c r="F42" s="28">
         <v>0.70138888888888884</v>
       </c>
-      <c r="G42" s="24">
+      <c r="G42" s="41">
         <v>4.166666666666663E-2</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" s="38" t="s">
+      <c r="A43" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B43" s="14" t="s">
+      <c r="B43" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="15">
+      <c r="C43" s="9">
         <v>46079</v>
       </c>
-      <c r="D43" s="16" t="s">
+      <c r="D43" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E43" s="17">
+      <c r="E43" s="29">
         <v>0.6875</v>
       </c>
-      <c r="F43" s="17">
+      <c r="F43" s="29">
         <v>0.84375</v>
       </c>
-      <c r="G43" s="18">
+      <c r="G43" s="38">
         <v>0.15625</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="38" t="s">
+      <c r="A44" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B44" s="25" t="s">
+      <c r="B44" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C44" s="26">
+      <c r="C44" s="15">
         <v>46079</v>
       </c>
-      <c r="D44" s="27" t="s">
+      <c r="D44" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="E44" s="28">
+      <c r="E44" s="30">
         <v>0.6875</v>
       </c>
-      <c r="F44" s="28">
+      <c r="F44" s="30">
         <v>0.84375</v>
       </c>
-      <c r="G44" s="29">
+      <c r="G44" s="39">
         <v>0.15625</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="39" t="s">
+      <c r="A45" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B45" s="33" t="s">
+      <c r="B45" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C45" s="5">
+      <c r="C45" s="3">
         <v>46079</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D45" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E45" s="7">
+      <c r="E45" s="27">
         <v>0.6875</v>
       </c>
-      <c r="F45" s="7">
+      <c r="F45" s="27">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G45" s="8">
+      <c r="G45" s="36">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="38" t="s">
+      <c r="A46" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="19" t="s">
+      <c r="B46" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C46" s="20">
+      <c r="C46" s="12">
         <v>46079</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="D46" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E46" s="22">
+      <c r="E46" s="28">
         <v>0.70833333333333337</v>
       </c>
-      <c r="F46" s="22">
+      <c r="F46" s="28">
         <v>0.83333333333333337</v>
       </c>
-      <c r="G46" s="24">
+      <c r="G46" s="41">
         <v>0.125</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" s="40" t="s">
+      <c r="A47" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B47" s="36" t="s">
+      <c r="B47" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C47" s="9">
+      <c r="C47" s="5">
         <v>46079</v>
       </c>
-      <c r="D47" s="10" t="s">
+      <c r="D47" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E47" s="11">
+      <c r="E47" s="31">
         <v>0.72916666666666663</v>
       </c>
-      <c r="F47" s="11">
+      <c r="F47" s="31">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G47" s="12">
+      <c r="G47" s="40">
         <v>0.125</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="38" t="s">
+      <c r="A48" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B48" s="33" t="s">
+      <c r="B48" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C48" s="5">
+      <c r="C48" s="3">
         <v>46080</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D48" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E48" s="7">
+      <c r="E48" s="27">
         <v>0.45833333333333331</v>
       </c>
-      <c r="F48" s="7">
+      <c r="F48" s="27">
         <v>0.5</v>
       </c>
-      <c r="G48" s="8">
+      <c r="G48" s="36">
         <v>4.1666666666666685E-2</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="39" t="s">
+      <c r="A49" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B49" s="25" t="s">
+      <c r="B49" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C49" s="26">
+      <c r="C49" s="15">
         <v>46080</v>
       </c>
-      <c r="D49" s="27" t="s">
+      <c r="D49" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E49" s="28">
+      <c r="E49" s="30">
         <v>0.59722222222222221</v>
       </c>
-      <c r="F49" s="28">
+      <c r="F49" s="30">
         <v>0.64930555555555558</v>
       </c>
-      <c r="G49" s="29">
+      <c r="G49" s="39">
         <v>5.208333333333337E-2</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A50" s="39" t="s">
+      <c r="A50" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B50" s="19" t="s">
+      <c r="B50" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C50" s="20">
+      <c r="C50" s="12">
         <v>46080</v>
       </c>
-      <c r="D50" s="21" t="s">
+      <c r="D50" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E50" s="22">
+      <c r="E50" s="28">
         <v>0.60416666666666663</v>
       </c>
-      <c r="F50" s="22">
+      <c r="F50" s="28">
         <v>0.65277777777777779</v>
       </c>
-      <c r="G50" s="24">
+      <c r="G50" s="41">
         <v>4.861111111111116E-2</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A51" s="39" t="s">
+      <c r="A51" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B51" s="14" t="s">
+      <c r="B51" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C51" s="15">
+      <c r="C51" s="9">
         <v>46080</v>
       </c>
-      <c r="D51" s="16" t="s">
+      <c r="D51" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E51" s="17">
+      <c r="E51" s="29">
         <v>0.63541666666666663</v>
       </c>
-      <c r="F51" s="17">
+      <c r="F51" s="29">
         <v>0.67708333333333337</v>
       </c>
-      <c r="G51" s="18">
+      <c r="G51" s="38">
         <v>4.1666666666666741E-2</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" s="38" t="s">
+      <c r="A52" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="19" t="s">
+      <c r="B52" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C52" s="20">
+      <c r="C52" s="12">
         <v>46080</v>
       </c>
-      <c r="D52" s="21" t="s">
+      <c r="D52" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="E52" s="22">
+      <c r="E52" s="28">
         <v>0.65277777777777779</v>
       </c>
-      <c r="F52" s="22">
+      <c r="F52" s="28">
         <v>0.70138888888888884</v>
       </c>
-      <c r="G52" s="24">
+      <c r="G52" s="41">
         <v>4.8611111111111049E-2</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" s="38" t="s">
+      <c r="A53" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="25" t="s">
+      <c r="B53" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C53" s="26">
+      <c r="C53" s="15">
         <v>46080</v>
       </c>
-      <c r="D53" s="27" t="s">
+      <c r="D53" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="E53" s="28">
+      <c r="E53" s="30">
         <v>0.65625</v>
       </c>
-      <c r="F53" s="28">
+      <c r="F53" s="30">
         <v>0.70833333333333337</v>
       </c>
-      <c r="G53" s="29">
+      <c r="G53" s="39">
         <v>5.208333333333337E-2</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A54" s="38" t="s">
+      <c r="A54" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B54" s="14" t="s">
+      <c r="B54" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C54" s="15">
+      <c r="C54" s="9">
         <v>46080</v>
       </c>
-      <c r="D54" s="16" t="s">
+      <c r="D54" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="E54" s="17">
+      <c r="E54" s="29">
         <v>0.6875</v>
       </c>
-      <c r="F54" s="17">
+      <c r="F54" s="29">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G54" s="18">
+      <c r="G54" s="38">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A55" s="39" t="s">
+      <c r="A55" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B55" s="33" t="s">
+      <c r="B55" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C55" s="5">
+      <c r="C55" s="3">
         <v>46080</v>
       </c>
-      <c r="D55" s="6" t="s">
+      <c r="D55" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E55" s="7">
+      <c r="E55" s="27">
         <v>0.6875</v>
       </c>
-      <c r="F55" s="7">
+      <c r="F55" s="27">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G55" s="8">
+      <c r="G55" s="36">
         <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A56" s="39" t="s">
+      <c r="A56" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B56" s="19" t="s">
+      <c r="B56" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C56" s="20">
+      <c r="C56" s="12">
         <v>46080</v>
       </c>
-      <c r="D56" s="21" t="s">
+      <c r="D56" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E56" s="22">
+      <c r="E56" s="28">
         <v>0.70833333333333337</v>
       </c>
-      <c r="F56" s="22">
+      <c r="F56" s="28">
         <v>0.83333333333333337</v>
       </c>
-      <c r="G56" s="24">
+      <c r="G56" s="41">
         <v>0.125</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" s="39" t="s">
+      <c r="A57" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B57" s="25" t="s">
+      <c r="B57" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C57" s="26">
+      <c r="C57" s="15">
         <v>46080</v>
       </c>
-      <c r="D57" s="27" t="s">
+      <c r="D57" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="E57" s="28">
+      <c r="E57" s="30">
         <v>0.71527777777777779</v>
       </c>
-      <c r="F57" s="28">
+      <c r="F57" s="30">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G57" s="29">
+      <c r="G57" s="39">
         <v>0.13888888888888884</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A58" s="40" t="s">
+      <c r="A58" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B58" s="36" t="s">
+      <c r="B58" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C58" s="9">
+      <c r="C58" s="5">
         <v>46080</v>
       </c>
-      <c r="D58" s="10" t="s">
+      <c r="D58" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E58" s="11">
+      <c r="E58" s="31">
         <v>0.72916666666666663</v>
       </c>
-      <c r="F58" s="11">
+      <c r="F58" s="31">
         <v>0.85416666666666663</v>
       </c>
-      <c r="G58" s="12">
+      <c r="G58" s="40">
         <v>0.125</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ultimo fichero de datos
</commit_message>
<xml_diff>
--- a/data/netejaS.xlsx
+++ b/data/netejaS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\_Flask_Python\gepV\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C13D1ED-9027-4C5E-8D84-39642FC2946B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5FAFCDF-82E8-4F24-8991-9F52EE365034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28692" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{E7BEF806-E2E7-45EE-9B5C-D08728AB8555}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="29">
   <si>
     <t>Nou Local Vigilant</t>
   </si>
@@ -114,6 +114,15 @@
   </si>
   <si>
     <t>El Caliu, jujats, espai jove. WC.</t>
+  </si>
+  <si>
+    <t>00NET</t>
+  </si>
+  <si>
+    <t>Escola Bressol</t>
+  </si>
+  <si>
+    <t>EURO</t>
   </si>
 </sst>
 </file>
@@ -124,7 +133,7 @@
     <numFmt numFmtId="164" formatCode="d\-m;@"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -170,8 +179,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -217,6 +234,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2CEEF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -270,7 +299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -334,6 +363,34 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="46" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="1" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="1" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="1" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -744,7 +801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67325F24-555F-4779-A203-C3E0DE13EEF4}">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
@@ -1720,8 +1777,216 @@
         <v>0.16666666666666663</v>
       </c>
     </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B43" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C43" s="31">
+        <v>46076</v>
+      </c>
+      <c r="D43" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E43" s="33">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="F43" s="33">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G43" s="34">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B44" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C44" s="31">
+        <v>46077</v>
+      </c>
+      <c r="D44" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E44" s="33">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="F44" s="33">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G44" s="34">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B45" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C45" s="31">
+        <v>46078</v>
+      </c>
+      <c r="D45" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E45" s="33">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="F45" s="33">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G45" s="34">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C46" s="31">
+        <v>46079</v>
+      </c>
+      <c r="D46" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E46" s="33">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="F46" s="33">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G46" s="34">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B47" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C47" s="31">
+        <v>46080</v>
+      </c>
+      <c r="D47" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E47" s="33">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="F47" s="33">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G47" s="34">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="B48" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48" s="37">
+        <v>46077</v>
+      </c>
+      <c r="D48" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="E48" s="39">
+        <v>0.6875</v>
+      </c>
+      <c r="F48" s="39">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G48" s="40">
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="B49" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C49" s="37">
+        <v>46078</v>
+      </c>
+      <c r="D49" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="E49" s="39">
+        <v>0.6875</v>
+      </c>
+      <c r="F49" s="39">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G49" s="40">
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="B50" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50" s="37">
+        <v>46079</v>
+      </c>
+      <c r="D50" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="E50" s="39">
+        <v>0.6875</v>
+      </c>
+      <c r="F50" s="39">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G50" s="40">
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="B51" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51" s="37">
+        <v>46080</v>
+      </c>
+      <c r="D51" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="E51" s="39">
+        <v>0.6875</v>
+      </c>
+      <c r="F51" s="39">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G51" s="40">
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <conditionalFormatting sqref="A2:A42">
+  <conditionalFormatting sqref="A2:A51">
     <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="00NET">
       <formula>NOT(ISERROR(SEARCH("00NET",A2)))</formula>
     </cfRule>

</xml_diff>

<commit_message>
Modificamos gitIgnore slsx, NO
</commit_message>
<xml_diff>
--- a/data/netejaS.xlsx
+++ b/data/netejaS.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\_Flask_Python\gepV\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5FAFCDF-82E8-4F24-8991-9F52EE365034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDB04844-5015-4AED-9F47-95AE5313AF2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28692" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{E7BEF806-E2E7-45EE-9B5C-D08728AB8555}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="WEB" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="30">
   <si>
     <t>Nou Local Vigilant</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>EURO</t>
+  </si>
+  <si>
+    <t>Escola VallgorguinaPRUEBA</t>
   </si>
 </sst>
 </file>
@@ -133,7 +136,7 @@
     <numFmt numFmtId="164" formatCode="d\-m;@"/>
     <numFmt numFmtId="165" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,6 +186,15 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="4" tint="-0.499984740745262"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -299,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -392,6 +404,9 @@
     </xf>
     <xf numFmtId="46" fontId="1" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -801,7 +816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67325F24-555F-4779-A203-C3E0DE13EEF4}">
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
@@ -1984,9 +1999,54 @@
         <v>0.16666666666666663</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="13.8" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="B52" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C52" s="41">
+        <v>46080</v>
+      </c>
+      <c r="D52" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="E52" s="39">
+        <v>0.6875</v>
+      </c>
+      <c r="F52" s="39">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G52" s="40">
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="B53" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53" s="37">
+        <v>46080</v>
+      </c>
+      <c r="D53" s="38" t="s">
+        <v>29</v>
+      </c>
+      <c r="E53" s="39">
+        <v>0.6875</v>
+      </c>
+      <c r="F53" s="39">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="G53" s="40">
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A51">
+  <conditionalFormatting sqref="A2:A53">
     <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="00NET">
       <formula>NOT(ISERROR(SEARCH("00NET",A2)))</formula>
     </cfRule>
@@ -2007,5 +2067,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>